<commit_message>
fix(docx/blank): declare common namespaces on <w:document> root
Real Word files declare the full Office namespace set (wps, wp, a, pic,
v, o, w10, ...) on <w:document>; OfficeCli's blank doc only declared
w/mc/w14. Subsequent raw-set injections referencing wps/wp/a (e.g. mc:Choice
Requires="wps" for DrawingML textboxes) failed MarkupCompatibility validation
because the prefix was not in scope at the AlternateContent element.

Mirror the LibreOffice docxexport MainXmlNamespaces() prefix set, and mark
only w14/wp14/w15 as mc:Ignorable (wps/wpg/wpi/wpc are gated by mc:Choice
fallback so they don't need it).

Regenerates examples/* docx outputs to pick up the new namespace block.
</commit_message>
<xml_diff>
--- a/examples/excel/charts-demo.xlsx
+++ b/examples/excel/charts-demo.xlsx
@@ -1030,7 +1030,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="Rc7972f3bf1d14dbb"/>
+          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R2d2f2dbc091b4dc6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1060,7 +1060,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R9fda1337d27d4851"/>
+          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R576f36af273242a2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1090,7 +1090,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R072548c96c004b93"/>
+          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R05b3ce2005f94eed"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1120,7 +1120,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="Rab5e11410f4e418a"/>
+          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="Rac9cf1de646d40dd"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1150,7 +1150,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R807d78cec5b14d11"/>
+          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R84aad00685b5475f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1180,7 +1180,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R743038bfe9cc46bc"/>
+          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="Rc18da4b2ae074cb0"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1414,6 +1414,6 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R978b7432b9214587"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0aec4e60af8d4980"/>
 </x:worksheet>
 </file>
</xml_diff>